<commit_message>
Update Unit Test Plan
</commit_message>
<xml_diff>
--- a/agile/Unit_Test_Plan_v0.1.xlsx
+++ b/agile/Unit_Test_Plan_v0.1.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\intelligent-bug-diagnosis-platform-internship\agile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B9D4FEA-5A3F-460B-9A40-165575443B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7190"/>
   </bookViews>
   <sheets>
     <sheet name="UT" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Actual Result</t>
   </si>
@@ -52,13 +51,150 @@
   </si>
   <si>
     <t>Sl: No:</t>
+  </si>
+  <si>
+    <t>Bug Report Submission</t>
+  </si>
+  <si>
+    <t>Bug File Upload</t>
+  </si>
+  <si>
+    <t>Triage Agent</t>
+  </si>
+  <si>
+    <t>Log Analysis Agent</t>
+  </si>
+  <si>
+    <t>Multi-Agent Orchestration</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Submit a bug through </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/bugs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Submit a bug containing a stack trace.</t>
+  </si>
+  <si>
+    <t>Submit a bug with an error such as NullPointerException.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Upload a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>.log</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> file through </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/bugs/upload</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Submit a bug report through </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/bugs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint.</t>
+    </r>
+  </si>
+  <si>
+    <t>Valid bug report data is provided.</t>
+  </si>
+  <si>
+    <t>Valid .log file is uploaded.</t>
+  </si>
+  <si>
+    <t>Bug report contains error information</t>
+  </si>
+  <si>
+    <t>Stack trace is available.</t>
+  </si>
+  <si>
+    <t>Valid bug submission</t>
+  </si>
+  <si>
+    <t>Bug report is accepted successfully</t>
+  </si>
+  <si>
+    <t>File is accepted and content is extracted.</t>
+  </si>
+  <si>
+    <t>Severity, priority and affected component are identified.</t>
+  </si>
+  <si>
+    <t>Exception type, failure point and affected code path are identified</t>
+  </si>
+  <si>
+    <t>Triage and Log Analysis outputs are combined as context.</t>
+  </si>
+  <si>
+    <t>Pass – Bug report submitted successfully.</t>
+  </si>
+  <si>
+    <t>Pass – File uploaded and content extracted successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Triage results generated successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Log analysis results generated successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Agent outputs combined successfully</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -78,6 +214,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -121,13 +262,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -442,18 +586,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="16.54296875" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -473,45 +617,105 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+    <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+    <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+    <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+    <row r="5" spans="1:6" ht="25" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+    <row r="6" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Unit Test Plan for Milestone 1 and Milestone 2
</commit_message>
<xml_diff>
--- a/agile/Unit_Test_Plan_v0.1.xlsx
+++ b/agile/Unit_Test_Plan_v0.1.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
   <si>
     <t>Actual Result</t>
   </si>
@@ -157,9 +157,6 @@
     <t>Stack trace is available.</t>
   </si>
   <si>
-    <t>Valid bug submission</t>
-  </si>
-  <si>
     <t>Bug report is accepted successfully</t>
   </si>
   <si>
@@ -188,6 +185,156 @@
   </si>
   <si>
     <t>Pass – Agent outputs combined successfully</t>
+  </si>
+  <si>
+    <t>Dataset Cleaning</t>
+  </si>
+  <si>
+    <t>Bug Report Chunking</t>
+  </si>
+  <si>
+    <t>Embedding Generation</t>
+  </si>
+  <si>
+    <t>Vector Store Indexing</t>
+  </si>
+  <si>
+    <t>Semantic Retrieval</t>
+  </si>
+  <si>
+    <t>Triage Confidence Scoring</t>
+  </si>
+  <si>
+    <t>Log Exception Identification</t>
+  </si>
+  <si>
+    <t>Log Failure Point Identification</t>
+  </si>
+  <si>
+    <t>Affected Code Path Identification</t>
+  </si>
+  <si>
+    <t>Agent Validation</t>
+  </si>
+  <si>
+    <t>Test Triage and Log Analysis with varied bug reports and error types.</t>
+  </si>
+  <si>
+    <t>Submit a bug containing code path information</t>
+  </si>
+  <si>
+    <t>Submit a stack trace containing a line number.</t>
+  </si>
+  <si>
+    <t>Submit a bug containing an exception in the stack trace.</t>
+  </si>
+  <si>
+    <t>Submit different types of bug reports to the Triage Agent.</t>
+  </si>
+  <si>
+    <t>Search for similar bugs using a sample bug description.</t>
+  </si>
+  <si>
+    <t>Store generated embeddings in FAISS.</t>
+  </si>
+  <si>
+    <t>Generate embeddings using Sentence</t>
+  </si>
+  <si>
+    <t>Apply chunking to historical bug reports.</t>
+  </si>
+  <si>
+    <t>Process Mozilla, Apache and Eclipse historical bug datasets.</t>
+  </si>
+  <si>
+    <t>Raw historical datasets are available.</t>
+  </si>
+  <si>
+    <t>Historical bug report data is available.</t>
+  </si>
+  <si>
+    <t>Valid bug report chunks are available.</t>
+  </si>
+  <si>
+    <t>Embeddings are available.</t>
+  </si>
+  <si>
+    <t>Similar historical bugs exist in the dataset.</t>
+  </si>
+  <si>
+    <t>Bug reports have different severity indicators.</t>
+  </si>
+  <si>
+    <t>Stack trace contains failure location.</t>
+  </si>
+  <si>
+    <t>Valid stack trace is provided.</t>
+  </si>
+  <si>
+    <t>Different bug formats and error types are provided</t>
+  </si>
+  <si>
+    <t>Stack trace contains an exception type.</t>
+  </si>
+  <si>
+    <t>Pass – Agents validated successfully with varied test cases.</t>
+  </si>
+  <si>
+    <t>Pass – Affected code path identified successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Failure point identified successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Confidence score and reasoning generated successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Relevant historical bugs retrieved successfully.</t>
+  </si>
+  <si>
+    <t>Pass – FAISS index created successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Embeddings generated successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Bug reports chunked successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Datasets cleaned and standardized successfully.</t>
+  </si>
+  <si>
+    <t>Pass – Exception type identified successfully.</t>
+  </si>
+  <si>
+    <t>Agents should return structured and relevant results.</t>
+  </si>
+  <si>
+    <t>Affected code path should be identified</t>
+  </si>
+  <si>
+    <t>Failure point should be identified.</t>
+  </si>
+  <si>
+    <t>Exception type should be identified</t>
+  </si>
+  <si>
+    <t>Confidence score and reasoning should be generated.</t>
+  </si>
+  <si>
+    <t>Relevant historical bugs should be retrieved.</t>
+  </si>
+  <si>
+    <t>FAISS vector index should be created.</t>
+  </si>
+  <si>
+    <t>Embeddings should be generated successfully.</t>
+  </si>
+  <si>
+    <t>Bug reports should be divided into meaningful chunks.</t>
+  </si>
+  <si>
+    <t>Dataset should be cleaned and standardized.</t>
   </si>
 </sst>
 </file>
@@ -235,7 +382,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -258,11 +405,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -272,6 +430,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.1796875" customWidth="1"/>
@@ -631,10 +792,10 @@
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -651,10 +812,10 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
@@ -671,10 +832,10 @@
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25" x14ac:dyDescent="0.25">
@@ -691,10 +852,10 @@
         <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="25" x14ac:dyDescent="0.35">
@@ -708,14 +869,217 @@
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>30</v>
       </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>